<commit_message>
updated progression tracking for m/w omnium and w mado
</commit_message>
<xml_diff>
--- a/pages/WR_progressions/Womens_Madison.xlsx
+++ b/pages/WR_progressions/Womens_Madison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\WR_progressions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4DA308-690C-4D1B-A425-477DA20B506B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0CF36B-ACE3-4F2C-975A-A570E04A121D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{8F2B8F41-998D-4BB8-BE11-A97939F5BC1E}"/>
   </bookViews>
@@ -457,17 +457,10 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -596,12 +589,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -609,26 +601,25 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -639,11 +630,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -699,6 +685,11 @@
           <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -1143,131 +1134,143 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="20">
+      <c r="B2" s="18">
         <v>2025</v>
       </c>
       <c r="C2" s="2">
         <v>45952</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="25">
+      <c r="H2" s="23">
         <v>22.484931506849314</v>
       </c>
-      <c r="I2" s="25">
+      <c r="I2" s="23">
         <v>31.635616438356163</v>
       </c>
-      <c r="J2" s="24">
+      <c r="J2" s="22">
         <v>1</v>
       </c>
-      <c r="K2" s="20">
-        <v>0</v>
-      </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20">
+      <c r="K2" s="18">
+        <v>0</v>
+      </c>
+      <c r="L2" s="18">
+        <v>8</v>
+      </c>
+      <c r="M2" s="18">
+        <v>2</v>
+      </c>
+      <c r="N2" s="18">
         <v>30</v>
       </c>
-      <c r="O2" s="20">
+      <c r="O2" s="18">
         <v>54.573</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B3" s="18">
         <v>2025</v>
       </c>
       <c r="C3" s="2">
         <v>45952</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="25">
+      <c r="H3" s="23">
         <v>25.2</v>
       </c>
-      <c r="I3" s="25">
+      <c r="I3" s="23">
         <v>27.92876712328767</v>
       </c>
-      <c r="J3" s="24">
+      <c r="J3" s="22">
         <v>2</v>
       </c>
-      <c r="K3" s="20">
-        <v>0</v>
-      </c>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20">
+      <c r="K3" s="18">
+        <v>0</v>
+      </c>
+      <c r="L3" s="18">
+        <v>8</v>
+      </c>
+      <c r="M3" s="18">
+        <v>3</v>
+      </c>
+      <c r="N3" s="18">
         <v>24</v>
       </c>
-      <c r="O3" s="20">
+      <c r="O3" s="18">
         <v>54.573</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="18">
         <v>2025</v>
       </c>
       <c r="C4" s="2">
         <v>45952</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="25">
+      <c r="H4" s="23">
         <v>26.347945205479451</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="23">
         <v>24.838356164383562</v>
       </c>
-      <c r="J4" s="24">
-        <v>3</v>
-      </c>
-      <c r="K4" s="20">
-        <v>0</v>
-      </c>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20">
+      <c r="J4" s="22">
+        <v>3</v>
+      </c>
+      <c r="K4" s="18">
+        <v>0</v>
+      </c>
+      <c r="L4" s="18">
+        <v>7</v>
+      </c>
+      <c r="M4" s="18">
+        <v>1</v>
+      </c>
+      <c r="N4" s="18">
         <v>20</v>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="18">
         <v>54.573</v>
       </c>
     </row>
@@ -1284,13 +1287,13 @@
       <c r="D5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="H5" s="3">
@@ -1299,16 +1302,22 @@
       <c r="I5" s="3">
         <v>24.216438356164385</v>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="22">
         <v>1</v>
       </c>
       <c r="K5">
         <v>20</v>
       </c>
+      <c r="L5">
+        <v>9</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
       <c r="N5">
         <v>53</v>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="4">
         <v>54.107999999999997</v>
       </c>
     </row>
@@ -1325,13 +1334,13 @@
       <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>19</v>
       </c>
       <c r="H6" s="3">
@@ -1340,16 +1349,22 @@
       <c r="I6" s="3">
         <v>25.717808219178082</v>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="22">
         <v>2</v>
       </c>
       <c r="K6">
         <v>20</v>
       </c>
+      <c r="L6">
+        <v>8</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
       <c r="N6">
         <v>43</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="4">
         <v>54.107999999999997</v>
       </c>
     </row>
@@ -1366,13 +1381,13 @@
       <c r="D7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>26</v>
       </c>
       <c r="H7" s="3">
@@ -1381,16 +1396,22 @@
       <c r="I7" s="3">
         <v>26.07123287671233</v>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="22">
         <v>3</v>
       </c>
       <c r="K7">
         <v>20</v>
       </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
       <c r="N7">
         <v>43</v>
       </c>
-      <c r="O7" s="5">
+      <c r="O7" s="4">
         <v>54.107999999999997</v>
       </c>
     </row>
@@ -1407,13 +1428,13 @@
       <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>20</v>
       </c>
       <c r="H8" s="3">
@@ -1422,11 +1443,17 @@
       <c r="I8" s="3">
         <v>32.290410958904111</v>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="22">
         <v>1</v>
       </c>
       <c r="K8">
         <v>20</v>
+      </c>
+      <c r="L8">
+        <v>9</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
       </c>
       <c r="N8">
         <v>46</v>
@@ -1448,13 +1475,13 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>30</v>
       </c>
       <c r="H9" s="3">
@@ -1463,11 +1490,17 @@
       <c r="I9" s="3">
         <v>26.920547945205481</v>
       </c>
-      <c r="J9" s="24">
+      <c r="J9" s="22">
         <v>2</v>
       </c>
       <c r="K9">
         <v>20</v>
+      </c>
+      <c r="L9">
+        <v>8</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
       </c>
       <c r="N9">
         <v>43</v>
@@ -1489,13 +1522,13 @@
       <c r="D10" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="3">
@@ -1504,11 +1537,17 @@
       <c r="I10" s="3">
         <v>30.627397260273973</v>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="22">
         <v>3</v>
       </c>
       <c r="K10">
         <v>0</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10">
+        <v>5</v>
       </c>
       <c r="N10">
         <v>42</v>
@@ -1530,13 +1569,13 @@
       <c r="D11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>23</v>
       </c>
       <c r="H11" s="3">
@@ -1545,11 +1584,17 @@
       <c r="I11" s="3">
         <v>23.717808219178082</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="22">
         <v>1</v>
       </c>
       <c r="K11">
         <v>20</v>
+      </c>
+      <c r="L11">
+        <v>4</v>
+      </c>
+      <c r="M11">
+        <v>3</v>
       </c>
       <c r="N11">
         <v>37</v>
@@ -1571,13 +1616,13 @@
       <c r="D12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H12" s="3">
@@ -1586,11 +1631,17 @@
       <c r="I12" s="3">
         <v>34.128767123287673</v>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="22">
         <v>2</v>
       </c>
       <c r="K12">
         <v>0</v>
+      </c>
+      <c r="L12">
+        <v>8</v>
+      </c>
+      <c r="M12">
+        <v>3</v>
       </c>
       <c r="N12">
         <v>31</v>
@@ -1612,13 +1663,13 @@
       <c r="D13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="3">
@@ -1627,11 +1678,17 @@
       <c r="I13" s="3">
         <v>20.621917808219177</v>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="22">
         <v>3</v>
       </c>
       <c r="K13">
         <v>20</v>
+      </c>
+      <c r="L13">
+        <v>3</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
       </c>
       <c r="N13">
         <v>28</v>
@@ -1653,13 +1710,13 @@
       <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H14" s="3">
@@ -1668,11 +1725,17 @@
       <c r="I14" s="3">
         <v>33.723287671232875</v>
       </c>
-      <c r="J14" s="8">
+      <c r="J14" s="7">
         <v>1</v>
       </c>
       <c r="K14">
         <v>0</v>
+      </c>
+      <c r="L14">
+        <v>9</v>
+      </c>
+      <c r="M14">
+        <v>5</v>
       </c>
       <c r="N14">
         <v>37</v>
@@ -1694,13 +1757,13 @@
       <c r="D15" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="7" t="s">
         <v>30</v>
       </c>
       <c r="H15" s="3">
@@ -1709,11 +1772,17 @@
       <c r="I15" s="3">
         <v>26.402739726027399</v>
       </c>
-      <c r="J15" s="8">
+      <c r="J15" s="7">
         <v>2</v>
       </c>
       <c r="K15">
         <v>0</v>
+      </c>
+      <c r="L15">
+        <v>7</v>
+      </c>
+      <c r="M15">
+        <v>2</v>
       </c>
       <c r="N15">
         <v>25</v>
@@ -1735,13 +1804,13 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="7" t="s">
         <v>69</v>
       </c>
       <c r="H16" s="3">
@@ -1750,11 +1819,17 @@
       <c r="I16" s="3">
         <v>29.824657534246576</v>
       </c>
-      <c r="J16" s="8">
+      <c r="J16" s="7">
         <v>3</v>
       </c>
       <c r="K16">
         <v>0</v>
+      </c>
+      <c r="L16">
+        <v>6</v>
+      </c>
+      <c r="M16">
+        <v>2</v>
       </c>
       <c r="N16">
         <v>19</v>
@@ -1776,13 +1851,13 @@
       <c r="D17" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="7" t="s">
         <v>72</v>
       </c>
       <c r="H17" s="3">
@@ -1791,11 +1866,17 @@
       <c r="I17" s="3">
         <v>22.186301369863013</v>
       </c>
-      <c r="J17" s="8">
+      <c r="J17" s="7">
         <v>1</v>
       </c>
       <c r="K17">
         <v>20</v>
+      </c>
+      <c r="L17">
+        <v>7</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
       </c>
       <c r="N17">
         <v>54</v>
@@ -1817,13 +1898,13 @@
       <c r="D18" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="7" t="s">
         <v>26</v>
       </c>
       <c r="H18" s="3">
@@ -1832,11 +1913,17 @@
       <c r="I18" s="3">
         <v>25.076712328767123</v>
       </c>
-      <c r="J18" s="8">
+      <c r="J18" s="7">
         <v>2</v>
       </c>
       <c r="K18">
         <v>20</v>
+      </c>
+      <c r="L18">
+        <v>10</v>
+      </c>
+      <c r="M18">
+        <v>4</v>
       </c>
       <c r="N18">
         <v>53</v>
@@ -1858,13 +1945,13 @@
       <c r="D19" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H19" s="3">
@@ -1873,11 +1960,17 @@
       <c r="I19" s="3">
         <v>20.139726027397259</v>
       </c>
-      <c r="J19" s="8">
+      <c r="J19" s="7">
         <v>3</v>
       </c>
       <c r="K19">
         <v>20</v>
+      </c>
+      <c r="L19">
+        <v>7</v>
+      </c>
+      <c r="M19">
+        <v>3</v>
       </c>
       <c r="N19">
         <v>49</v>
@@ -1899,13 +1992,13 @@
       <c r="D20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H20" s="3">
@@ -1914,11 +2007,17 @@
       <c r="I20" s="3">
         <v>29.427397260273974</v>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="22">
         <v>1</v>
       </c>
       <c r="K20">
         <v>0</v>
+      </c>
+      <c r="L20">
+        <v>7</v>
+      </c>
+      <c r="M20">
+        <v>5</v>
       </c>
       <c r="N20">
         <v>31</v>
@@ -1940,13 +2039,13 @@
       <c r="D21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="7" t="s">
         <v>42</v>
       </c>
       <c r="H21" s="3">
@@ -1955,11 +2054,17 @@
       <c r="I21" s="3">
         <v>27.950684931506849</v>
       </c>
-      <c r="J21" s="24">
+      <c r="J21" s="22">
         <v>2</v>
       </c>
       <c r="K21">
         <v>0</v>
+      </c>
+      <c r="L21">
+        <v>8</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
       </c>
       <c r="N21">
         <v>27</v>
@@ -1981,13 +2086,13 @@
       <c r="D22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="7" t="s">
         <v>69</v>
       </c>
       <c r="H22" s="3">
@@ -1996,11 +2101,17 @@
       <c r="I22" s="3">
         <v>29.632876712328766</v>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="22">
         <v>3</v>
       </c>
       <c r="K22">
         <v>0</v>
+      </c>
+      <c r="L22">
+        <v>8</v>
+      </c>
+      <c r="M22">
+        <v>2</v>
       </c>
       <c r="N22">
         <v>23</v>
@@ -2010,25 +2121,25 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="17">
+      <c r="B23" s="15">
         <v>2023</v>
       </c>
       <c r="C23" s="2">
         <v>45146</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="8" t="s" cm="1">
+      <c r="E23" s="7" t="s" cm="1">
         <v>62</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H23" s="3">
@@ -2037,11 +2148,17 @@
       <c r="I23" s="3">
         <v>28.926027397260274</v>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="22">
         <v>1</v>
       </c>
-      <c r="K23" s="4">
-        <v>0</v>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23">
+        <v>3</v>
       </c>
       <c r="N23">
         <v>28</v>
@@ -2051,25 +2168,25 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="17">
+      <c r="B24" s="15">
         <v>2023</v>
       </c>
       <c r="C24" s="2">
         <v>45146</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E24" s="8" t="s" cm="1">
+      <c r="E24" s="7" t="s" cm="1">
         <v>76</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="7" t="s">
         <v>42</v>
       </c>
       <c r="H24" s="3">
@@ -2078,11 +2195,17 @@
       <c r="I24" s="3">
         <v>27.449315068493149</v>
       </c>
-      <c r="J24" s="24">
+      <c r="J24" s="22">
         <v>2</v>
       </c>
-      <c r="K24" s="4">
-        <v>0</v>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>7</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
       </c>
       <c r="N24">
         <v>25</v>
@@ -2092,25 +2215,25 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="17">
+      <c r="B25" s="15">
         <v>2023</v>
       </c>
       <c r="C25" s="2">
         <v>45146</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="8" t="s" cm="1">
+      <c r="E25" s="7" t="s" cm="1">
         <v>51</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="7" t="s">
         <v>30</v>
       </c>
       <c r="H25" s="3">
@@ -2119,11 +2242,17 @@
       <c r="I25" s="3">
         <v>24.575342465753426</v>
       </c>
-      <c r="J25" s="24">
-        <v>3</v>
-      </c>
-      <c r="K25" s="4">
-        <v>0</v>
+      <c r="J25" s="22">
+        <v>3</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>6</v>
+      </c>
+      <c r="M25">
+        <v>2</v>
       </c>
       <c r="N25">
         <v>22</v>
@@ -2145,13 +2274,13 @@
       <c r="D26" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H26" s="3">
@@ -2160,11 +2289,17 @@
       <c r="I26" s="3">
         <v>27.463013698630139</v>
       </c>
-      <c r="J26" s="24">
+      <c r="J26" s="22">
         <v>1</v>
       </c>
       <c r="K26">
         <v>20</v>
+      </c>
+      <c r="L26">
+        <v>9</v>
+      </c>
+      <c r="M26">
+        <v>3</v>
       </c>
       <c r="N26">
         <v>53</v>
@@ -2186,13 +2321,13 @@
       <c r="D27" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H27" s="3">
@@ -2201,11 +2336,17 @@
       <c r="I27" s="3">
         <v>32.742465753424661</v>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="22">
         <v>2</v>
       </c>
       <c r="K27">
         <v>20</v>
+      </c>
+      <c r="L27">
+        <v>8</v>
+      </c>
+      <c r="M27">
+        <v>2</v>
       </c>
       <c r="N27">
         <v>44</v>
@@ -2227,13 +2368,13 @@
       <c r="D28" t="s">
         <v>14</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G28" s="7" t="s">
         <v>23</v>
       </c>
       <c r="H28" s="3">
@@ -2242,11 +2383,17 @@
       <c r="I28" s="3">
         <v>23.473972602739725</v>
       </c>
-      <c r="J28" s="24">
+      <c r="J28" s="22">
         <v>3</v>
       </c>
       <c r="K28">
         <v>20</v>
+      </c>
+      <c r="L28">
+        <v>6</v>
+      </c>
+      <c r="M28">
+        <v>3</v>
       </c>
       <c r="N28">
         <v>41</v>
@@ -2262,19 +2409,19 @@
       <c r="B29" s="1">
         <v>2023</v>
       </c>
-      <c r="C29" s="18">
+      <c r="C29" s="16">
         <v>45002</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="F29" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="G29" s="13" t="s">
+      <c r="G29" s="11" t="s">
         <v>30</v>
       </c>
       <c r="H29" s="3">
@@ -2283,16 +2430,22 @@
       <c r="I29" s="3">
         <v>23.906849315068492</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="11">
         <v>1</v>
       </c>
-      <c r="K29" s="4">
-        <v>0</v>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>10</v>
+      </c>
+      <c r="M29">
+        <v>4</v>
       </c>
       <c r="N29">
         <v>35</v>
       </c>
-      <c r="O29" s="7">
+      <c r="O29" s="6">
         <v>50.966999999999999</v>
       </c>
     </row>
@@ -2303,19 +2456,19 @@
       <c r="B30" s="1">
         <v>2023</v>
       </c>
-      <c r="C30" s="18">
+      <c r="C30" s="16">
         <v>45002</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="13" t="s">
+      <c r="G30" s="11" t="s">
         <v>20</v>
       </c>
       <c r="H30" s="3">
@@ -2324,16 +2477,22 @@
       <c r="I30" s="3">
         <v>30.69041095890411</v>
       </c>
-      <c r="J30" s="13">
+      <c r="J30" s="11">
         <v>2</v>
       </c>
       <c r="K30">
         <v>0</v>
+      </c>
+      <c r="L30">
+        <v>8</v>
+      </c>
+      <c r="M30">
+        <v>3</v>
       </c>
       <c r="N30">
         <v>34</v>
       </c>
-      <c r="O30" s="7">
+      <c r="O30" s="6">
         <v>50.966999999999999</v>
       </c>
     </row>
@@ -2344,19 +2503,19 @@
       <c r="B31" s="1">
         <v>2023</v>
       </c>
-      <c r="C31" s="18">
+      <c r="C31" s="16">
         <v>45002</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F31" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="G31" s="13" t="s">
+      <c r="G31" s="11" t="s">
         <v>26</v>
       </c>
       <c r="H31" s="3">
@@ -2365,16 +2524,22 @@
       <c r="I31" s="3">
         <v>22.205479452054796</v>
       </c>
-      <c r="J31" s="13">
+      <c r="J31" s="11">
         <v>3</v>
       </c>
       <c r="K31">
         <v>0</v>
+      </c>
+      <c r="L31">
+        <v>8</v>
+      </c>
+      <c r="M31">
+        <v>3</v>
       </c>
       <c r="N31">
         <v>24</v>
       </c>
-      <c r="O31" s="7">
+      <c r="O31" s="6">
         <v>50.966999999999999</v>
       </c>
     </row>
@@ -2391,13 +2556,13 @@
       <c r="D32" t="s">
         <v>14</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="G32" s="21" t="s">
+      <c r="G32" s="19" t="s">
         <v>20</v>
       </c>
       <c r="H32" s="3">
@@ -2406,11 +2571,17 @@
       <c r="I32" s="3">
         <v>30.641095890410959</v>
       </c>
-      <c r="J32" s="24">
+      <c r="J32" s="22">
         <v>1</v>
       </c>
       <c r="K32">
         <v>20</v>
+      </c>
+      <c r="L32">
+        <v>8</v>
+      </c>
+      <c r="M32">
+        <v>2</v>
       </c>
       <c r="N32">
         <v>42</v>
@@ -2432,13 +2603,13 @@
       <c r="D33" t="s">
         <v>14</v>
       </c>
-      <c r="E33" s="21" t="s">
+      <c r="E33" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="19" t="s">
         <v>30</v>
       </c>
       <c r="H33" s="3">
@@ -2447,11 +2618,17 @@
       <c r="I33" s="3">
         <v>25.271232876712329</v>
       </c>
-      <c r="J33" s="24">
+      <c r="J33" s="22">
         <v>2</v>
       </c>
       <c r="K33">
         <v>0</v>
+      </c>
+      <c r="L33">
+        <v>10</v>
+      </c>
+      <c r="M33">
+        <v>3</v>
       </c>
       <c r="N33">
         <v>32</v>
@@ -2473,13 +2650,13 @@
       <c r="D34" t="s">
         <v>14</v>
       </c>
-      <c r="E34" s="21" t="s">
+      <c r="E34" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="19" t="s">
         <v>23</v>
       </c>
       <c r="H34" s="3">
@@ -2488,11 +2665,17 @@
       <c r="I34" s="3">
         <v>22.997260273972604</v>
       </c>
-      <c r="J34" s="24">
+      <c r="J34" s="22">
         <v>3</v>
       </c>
       <c r="K34">
         <v>0</v>
+      </c>
+      <c r="L34">
+        <v>6</v>
+      </c>
+      <c r="M34">
+        <v>3</v>
       </c>
       <c r="N34">
         <v>26</v>
@@ -2514,13 +2697,13 @@
       <c r="D35" t="s">
         <v>18</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F35" s="13" t="s">
+      <c r="F35" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="G35" s="13" t="s">
+      <c r="G35" s="11" t="s">
         <v>16</v>
       </c>
       <c r="H35" s="3">
@@ -2529,16 +2712,22 @@
       <c r="I35" s="3">
         <v>26.947945205479453</v>
       </c>
-      <c r="J35" s="24">
+      <c r="J35" s="22">
         <v>1</v>
       </c>
       <c r="K35">
         <v>20</v>
       </c>
+      <c r="L35">
+        <v>3</v>
+      </c>
+      <c r="M35">
+        <v>2</v>
+      </c>
       <c r="N35">
         <v>32</v>
       </c>
-      <c r="O35" s="7">
+      <c r="O35" s="6">
         <v>53.28</v>
       </c>
     </row>
@@ -2555,13 +2744,13 @@
       <c r="D36" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F36" s="13" t="s">
+      <c r="F36" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="G36" s="13" t="s">
+      <c r="G36" s="11" t="s">
         <v>30</v>
       </c>
       <c r="H36" s="3">
@@ -2570,16 +2759,22 @@
       <c r="I36" s="3">
         <v>23.493150684931507</v>
       </c>
-      <c r="J36" s="24">
+      <c r="J36" s="22">
         <v>2</v>
       </c>
       <c r="K36">
         <v>0</v>
+      </c>
+      <c r="L36">
+        <v>9</v>
+      </c>
+      <c r="M36">
+        <v>2</v>
       </c>
       <c r="N36">
         <v>31</v>
       </c>
-      <c r="O36" s="7">
+      <c r="O36" s="6">
         <v>53.28</v>
       </c>
     </row>
@@ -2596,13 +2791,13 @@
       <c r="D37" t="s">
         <v>18</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G37" s="13" t="s">
+      <c r="G37" s="11" t="s">
         <v>20</v>
       </c>
       <c r="H37" s="3">
@@ -2611,16 +2806,22 @@
       <c r="I37" s="3">
         <v>30.276712328767122</v>
       </c>
-      <c r="J37" s="24">
+      <c r="J37" s="22">
         <v>3</v>
       </c>
       <c r="K37">
         <v>0</v>
+      </c>
+      <c r="L37">
+        <v>7</v>
+      </c>
+      <c r="M37">
+        <v>2</v>
       </c>
       <c r="N37">
         <v>23</v>
       </c>
-      <c r="O37" s="7">
+      <c r="O37" s="6">
         <v>53.28</v>
       </c>
     </row>
@@ -2637,13 +2838,13 @@
       <c r="D38" t="s">
         <v>14</v>
       </c>
-      <c r="E38" s="21" t="s">
+      <c r="E38" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="F38" s="21" t="s">
+      <c r="F38" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G38" s="22" t="s">
+      <c r="G38" s="20" t="s">
         <v>69</v>
       </c>
       <c r="H38" s="3">
@@ -2652,11 +2853,17 @@
       <c r="I38" s="3">
         <v>27.561643835616437</v>
       </c>
-      <c r="J38" s="24">
+      <c r="J38" s="22">
         <v>1</v>
       </c>
       <c r="K38">
         <v>0</v>
+      </c>
+      <c r="L38">
+        <v>11</v>
+      </c>
+      <c r="M38">
+        <v>7</v>
       </c>
       <c r="N38">
         <v>48</v>
@@ -2678,13 +2885,13 @@
       <c r="D39" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="21" t="s">
+      <c r="E39" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="F39" s="21" t="s">
+      <c r="F39" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="G39" s="22" t="s">
+      <c r="G39" s="20" t="s">
         <v>23</v>
       </c>
       <c r="H39" s="3">
@@ -2693,11 +2900,17 @@
       <c r="I39" s="3">
         <v>22.983561643835618</v>
       </c>
-      <c r="J39" s="24">
+      <c r="J39" s="22">
         <v>2</v>
       </c>
       <c r="K39">
         <v>0</v>
+      </c>
+      <c r="L39">
+        <v>10</v>
+      </c>
+      <c r="M39">
+        <v>2</v>
       </c>
       <c r="N39">
         <v>35</v>
@@ -2719,13 +2932,13 @@
       <c r="D40" t="s">
         <v>14</v>
       </c>
-      <c r="E40" s="21" t="s">
+      <c r="E40" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="F40" s="21" t="s">
+      <c r="F40" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="G40" s="22" t="s">
+      <c r="G40" s="20" t="s">
         <v>26</v>
       </c>
       <c r="H40" s="3">
@@ -2734,11 +2947,17 @@
       <c r="I40" s="3">
         <v>19.86849315068493</v>
       </c>
-      <c r="J40" s="24">
-        <v>3</v>
-      </c>
-      <c r="K40" s="4">
-        <v>0</v>
+      <c r="J40" s="22">
+        <v>3</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+      <c r="L40">
+        <v>10</v>
+      </c>
+      <c r="M40">
+        <v>1</v>
       </c>
       <c r="N40">
         <v>29</v>
@@ -2760,13 +2979,13 @@
       <c r="D41" t="s">
         <v>14</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="F41" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="23" t="s">
+      <c r="G41" s="21" t="s">
         <v>23</v>
       </c>
       <c r="H41" s="3">
@@ -2775,11 +2994,17 @@
       <c r="I41" s="3">
         <v>22.906849315068492</v>
       </c>
-      <c r="J41" s="24">
+      <c r="J41" s="22">
         <v>1</v>
       </c>
       <c r="K41">
         <v>20</v>
+      </c>
+      <c r="L41">
+        <v>9</v>
+      </c>
+      <c r="M41">
+        <v>5</v>
       </c>
       <c r="N41">
         <v>54</v>
@@ -2801,13 +3026,13 @@
       <c r="D42" t="s">
         <v>14</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="F42" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="G42" s="23" t="s">
+      <c r="G42" s="21" t="s">
         <v>42</v>
       </c>
       <c r="H42" s="3">
@@ -2816,11 +3041,17 @@
       <c r="I42" s="3">
         <v>23.509589041095889</v>
       </c>
-      <c r="J42" s="24">
+      <c r="J42" s="22">
         <v>2</v>
       </c>
       <c r="K42">
         <v>20</v>
+      </c>
+      <c r="L42">
+        <v>6</v>
+      </c>
+      <c r="M42">
+        <v>3</v>
       </c>
       <c r="N42">
         <v>45</v>
@@ -2842,13 +3073,13 @@
       <c r="D43" t="s">
         <v>14</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="F43" s="13" t="s">
+      <c r="F43" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G43" s="23" t="s">
+      <c r="G43" s="21" t="s">
         <v>93</v>
       </c>
       <c r="H43" s="3">
@@ -2857,11 +3088,17 @@
       <c r="I43" s="3">
         <v>28.052054794520547</v>
       </c>
-      <c r="J43" s="24">
+      <c r="J43" s="22">
         <v>3</v>
       </c>
       <c r="K43">
         <v>20</v>
+      </c>
+      <c r="L43">
+        <v>5</v>
+      </c>
+      <c r="M43">
+        <v>0</v>
       </c>
       <c r="N43">
         <v>29</v>
@@ -2883,13 +3120,13 @@
       <c r="D44" t="s">
         <v>14</v>
       </c>
-      <c r="E44" s="21" t="s">
+      <c r="E44" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="F44" s="21" t="s">
+      <c r="F44" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G44" s="22" t="s">
+      <c r="G44" s="20" t="s">
         <v>30</v>
       </c>
       <c r="H44" s="3">
@@ -2898,11 +3135,17 @@
       <c r="I44" s="3">
         <v>23.016438356164382</v>
       </c>
-      <c r="J44" s="24">
+      <c r="J44" s="22">
         <v>1</v>
       </c>
       <c r="K44">
         <v>0</v>
+      </c>
+      <c r="L44">
+        <v>8</v>
+      </c>
+      <c r="M44">
+        <v>5</v>
       </c>
       <c r="N44">
         <v>33</v>
@@ -2924,13 +3167,13 @@
       <c r="D45" t="s">
         <v>14</v>
       </c>
-      <c r="E45" s="21" t="s">
+      <c r="E45" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="F45" s="21" t="s">
+      <c r="F45" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="G45" s="22" t="s">
+      <c r="G45" s="20" t="s">
         <v>23</v>
       </c>
       <c r="H45" s="3">
@@ -2939,11 +3182,17 @@
       <c r="I45" s="3">
         <v>21.339726027397262</v>
       </c>
-      <c r="J45" s="24">
+      <c r="J45" s="22">
         <v>2</v>
       </c>
       <c r="K45">
         <v>0</v>
+      </c>
+      <c r="L45">
+        <v>7</v>
+      </c>
+      <c r="M45">
+        <v>1</v>
       </c>
       <c r="N45">
         <v>23</v>
@@ -2965,13 +3214,13 @@
       <c r="D46" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="21" t="s">
+      <c r="E46" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F46" s="21" t="s">
+      <c r="F46" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="G46" s="22" t="s">
+      <c r="G46" s="20" t="s">
         <v>20</v>
       </c>
       <c r="H46" s="3">
@@ -2980,11 +3229,17 @@
       <c r="I46" s="3">
         <v>29.8</v>
       </c>
-      <c r="J46" s="24">
+      <c r="J46" s="22">
         <v>3</v>
       </c>
       <c r="K46">
         <v>0</v>
+      </c>
+      <c r="L46">
+        <v>6</v>
+      </c>
+      <c r="M46">
+        <v>1</v>
       </c>
       <c r="N46">
         <v>18</v>
@@ -3006,13 +3261,13 @@
       <c r="D47" t="s">
         <v>18</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F47" s="6" t="s">
+      <c r="F47" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G47" s="6" t="s">
+      <c r="G47" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H47" s="3">
@@ -3021,11 +3276,17 @@
       <c r="I47" s="3">
         <v>39.049315068493151</v>
       </c>
-      <c r="J47" s="7">
+      <c r="J47" s="6">
         <v>1</v>
       </c>
       <c r="K47">
         <v>0</v>
+      </c>
+      <c r="L47">
+        <v>9</v>
+      </c>
+      <c r="M47">
+        <v>4</v>
       </c>
       <c r="N47">
         <v>35</v>
@@ -3047,13 +3308,13 @@
       <c r="D48" t="s">
         <v>18</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E48" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F48" s="6" t="s">
+      <c r="F48" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="G48" s="5" t="s">
         <v>30</v>
       </c>
       <c r="H48" s="3">
@@ -3062,11 +3323,17 @@
       <c r="I48" s="3">
         <v>21.758904109589039</v>
       </c>
-      <c r="J48" s="7">
+      <c r="J48" s="6">
         <v>2</v>
       </c>
       <c r="K48">
         <v>0</v>
+      </c>
+      <c r="L48">
+        <v>9</v>
+      </c>
+      <c r="M48">
+        <v>2</v>
       </c>
       <c r="N48">
         <v>30</v>
@@ -3076,25 +3343,25 @@
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A49" s="8" t="s">
+      <c r="A49" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B49" s="8">
+      <c r="B49" s="7">
         <v>2021</v>
       </c>
-      <c r="C49" s="9">
+      <c r="C49" s="8">
         <v>44493</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D49" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E49" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F49" s="6" t="s">
+      <c r="F49" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G49" s="6" t="s">
+      <c r="G49" s="5" t="s">
         <v>28</v>
       </c>
       <c r="H49" s="3">
@@ -3103,11 +3370,17 @@
       <c r="I49" s="3">
         <v>31.24931506849315</v>
       </c>
-      <c r="J49" s="7">
+      <c r="J49" s="6">
         <v>3</v>
       </c>
       <c r="K49">
         <v>0</v>
+      </c>
+      <c r="L49">
+        <v>10</v>
+      </c>
+      <c r="M49">
+        <v>1</v>
       </c>
       <c r="N49">
         <v>24</v>
@@ -3117,16 +3390,16 @@
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B50" s="8">
+      <c r="B50" s="7">
         <v>2021</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="8">
         <v>44450</v>
       </c>
-      <c r="D50" s="8" t="s">
+      <c r="D50" s="7" t="s">
         <v>14</v>
       </c>
       <c r="E50" s="1" t="s">
@@ -3144,11 +3417,17 @@
       <c r="I50" s="3">
         <v>23.252054794520546</v>
       </c>
-      <c r="J50" s="7">
+      <c r="J50" s="6">
         <v>1</v>
       </c>
       <c r="K50">
         <v>0</v>
+      </c>
+      <c r="L50">
+        <v>11</v>
+      </c>
+      <c r="M50">
+        <v>10</v>
       </c>
       <c r="N50">
         <v>53</v>
@@ -3158,16 +3437,16 @@
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="7">
         <v>2021</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="8">
         <v>44450</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="D51" s="7" t="s">
         <v>14</v>
       </c>
       <c r="E51" s="1" t="s">
@@ -3185,10 +3464,16 @@
       <c r="I51" s="3">
         <v>27.358904109589041</v>
       </c>
-      <c r="J51" s="7">
+      <c r="J51" s="6">
         <v>2</v>
       </c>
       <c r="K51">
+        <v>0</v>
+      </c>
+      <c r="L51">
+        <v>9</v>
+      </c>
+      <c r="M51">
         <v>0</v>
       </c>
       <c r="N51">
@@ -3199,16 +3484,16 @@
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A52" s="10" t="s">
+      <c r="A52" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="9">
         <v>2021</v>
       </c>
-      <c r="C52" s="11">
+      <c r="C52" s="10">
         <v>44450</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="9" t="s">
         <v>14</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -3226,10 +3511,16 @@
       <c r="I52" s="3">
         <v>20.873972602739727</v>
       </c>
-      <c r="J52" s="7">
-        <v>3</v>
-      </c>
-      <c r="K52" s="12">
+      <c r="J52" s="6">
+        <v>3</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+      <c r="L52">
+        <v>10</v>
+      </c>
+      <c r="M52">
         <v>0</v>
       </c>
       <c r="N52">
@@ -3240,16 +3531,16 @@
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A53" s="13" t="s">
+      <c r="A53" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B53" s="13">
+      <c r="B53" s="11">
         <v>2021</v>
       </c>
-      <c r="C53" s="14">
+      <c r="C53" s="12">
         <v>44415</v>
       </c>
-      <c r="D53" s="13" t="s">
+      <c r="D53" s="11" t="s">
         <v>22</v>
       </c>
       <c r="E53" t="s">
@@ -3267,30 +3558,36 @@
       <c r="I53" s="3">
         <v>29.304109589041097</v>
       </c>
-      <c r="J53" s="6">
+      <c r="J53" s="5">
         <v>1</v>
       </c>
-      <c r="K53" s="13">
+      <c r="K53" s="11">
         <v>20</v>
       </c>
-      <c r="N53" s="13">
+      <c r="L53">
+        <v>12</v>
+      </c>
+      <c r="M53">
+        <v>10</v>
+      </c>
+      <c r="N53" s="11">
         <v>78</v>
       </c>
-      <c r="O53" s="7">
+      <c r="O53" s="6">
         <v>54.947000000000003</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A54" s="13" t="s">
+      <c r="A54" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B54" s="13">
+      <c r="B54" s="11">
         <v>2021</v>
       </c>
-      <c r="C54" s="14">
+      <c r="C54" s="12">
         <v>44415</v>
       </c>
-      <c r="D54" s="13" t="s">
+      <c r="D54" s="11" t="s">
         <v>22</v>
       </c>
       <c r="E54" t="s">
@@ -3308,30 +3605,36 @@
       <c r="I54" s="3">
         <v>29.084931506849315</v>
       </c>
-      <c r="J54" s="6">
+      <c r="J54" s="5">
         <v>2</v>
       </c>
-      <c r="K54" s="13">
+      <c r="K54" s="11">
         <v>20</v>
       </c>
-      <c r="N54" s="13">
+      <c r="L54">
+        <v>7</v>
+      </c>
+      <c r="M54">
+        <v>0</v>
+      </c>
+      <c r="N54" s="11">
         <v>35</v>
       </c>
-      <c r="O54" s="7">
+      <c r="O54" s="6">
         <v>54.947000000000003</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A55" s="13" t="s">
+      <c r="A55" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B55" s="13">
+      <c r="B55" s="11">
         <v>2021</v>
       </c>
-      <c r="C55" s="14">
+      <c r="C55" s="12">
         <v>44415</v>
       </c>
-      <c r="D55" s="13" t="s">
+      <c r="D55" s="11" t="s">
         <v>22</v>
       </c>
       <c r="E55" t="s">
@@ -3349,39 +3652,45 @@
       <c r="I55" s="3">
         <v>22.041095890410958</v>
       </c>
-      <c r="J55" s="6">
-        <v>3</v>
-      </c>
-      <c r="K55" s="13">
+      <c r="J55" s="5">
+        <v>3</v>
+      </c>
+      <c r="K55" s="11">
         <v>20</v>
       </c>
-      <c r="N55" s="13">
+      <c r="L55">
+        <v>3</v>
+      </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+      <c r="N55" s="11">
         <v>26</v>
       </c>
-      <c r="O55" s="7">
+      <c r="O55" s="6">
         <v>54.947000000000003</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A56" s="15" t="s">
+      <c r="A56" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B56" s="15">
+      <c r="B56" s="13">
         <v>2021</v>
       </c>
       <c r="C56" s="2">
         <v>44387</v>
       </c>
-      <c r="D56" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E56" s="6" t="s">
+      <c r="D56" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="F56" s="6" t="s">
+      <c r="F56" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="G56" s="6" t="s">
+      <c r="G56" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H56" s="3">
@@ -3390,11 +3699,17 @@
       <c r="I56" s="3">
         <v>24.772602739726029</v>
       </c>
-      <c r="J56" s="7">
+      <c r="J56" s="6">
         <v>1</v>
       </c>
       <c r="K56">
         <v>0</v>
+      </c>
+      <c r="L56">
+        <v>12</v>
+      </c>
+      <c r="M56">
+        <v>7</v>
       </c>
       <c r="N56">
         <v>50</v>
@@ -3404,25 +3719,25 @@
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="15">
+      <c r="B57" s="13">
         <v>2021</v>
       </c>
       <c r="C57" s="2">
         <v>44387</v>
       </c>
-      <c r="D57" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E57" s="6" t="s">
+      <c r="D57" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E57" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="F57" s="6" t="s">
+      <c r="F57" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G57" s="6" t="s">
+      <c r="G57" s="5" t="s">
         <v>38</v>
       </c>
       <c r="H57" s="3">
@@ -3431,11 +3746,17 @@
       <c r="I57" s="3">
         <v>17.663013698630138</v>
       </c>
-      <c r="J57" s="7">
+      <c r="J57" s="6">
         <v>2</v>
       </c>
       <c r="K57">
         <v>0</v>
+      </c>
+      <c r="L57">
+        <v>11</v>
+      </c>
+      <c r="M57">
+        <v>4</v>
       </c>
       <c r="N57">
         <v>41</v>
@@ -3445,25 +3766,25 @@
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A58" s="15" t="s">
+      <c r="A58" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="15">
+      <c r="B58" s="13">
         <v>2021</v>
       </c>
       <c r="C58" s="2">
         <v>44387</v>
       </c>
-      <c r="D58" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E58" s="6" t="s">
+      <c r="D58" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E58" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F58" s="6" t="s">
+      <c r="F58" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G58" s="6" t="s">
+      <c r="G58" s="5" t="s">
         <v>114</v>
       </c>
       <c r="H58" s="3">
@@ -3472,11 +3793,17 @@
       <c r="I58" s="3">
         <v>24.142465753424659</v>
       </c>
-      <c r="J58" s="7">
-        <v>3</v>
-      </c>
-      <c r="K58" s="4">
-        <v>0</v>
+      <c r="J58" s="6">
+        <v>3</v>
+      </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
+      <c r="L58">
+        <v>12</v>
+      </c>
+      <c r="M58">
+        <v>1</v>
       </c>
       <c r="N58">
         <v>32</v>
@@ -3486,16 +3813,16 @@
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B59" s="8">
+      <c r="B59" s="7">
         <v>2020</v>
       </c>
-      <c r="C59" s="9">
+      <c r="C59" s="8">
         <v>43891</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E59" s="1" t="s">
@@ -3513,30 +3840,36 @@
       <c r="I59" s="3">
         <v>28.767123287671232</v>
       </c>
-      <c r="J59" s="7">
+      <c r="J59" s="6">
         <v>1</v>
       </c>
       <c r="K59">
         <v>0</v>
+      </c>
+      <c r="L59">
+        <v>11</v>
+      </c>
+      <c r="M59">
+        <v>3</v>
       </c>
       <c r="N59">
         <v>36</v>
       </c>
-      <c r="O59" s="6">
+      <c r="O59" s="5">
         <v>50.908000000000001</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A60" s="8" t="s">
+      <c r="A60" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B60" s="8">
+      <c r="B60" s="7">
         <v>2020</v>
       </c>
-      <c r="C60" s="9">
+      <c r="C60" s="8">
         <v>43891</v>
       </c>
-      <c r="D60" s="8" t="s">
+      <c r="D60" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E60" s="1" t="s">
@@ -3554,30 +3887,36 @@
       <c r="I60" s="3">
         <v>20.109589041095891</v>
       </c>
-      <c r="J60" s="7">
+      <c r="J60" s="6">
         <v>2</v>
       </c>
-      <c r="K60" s="4">
-        <v>0</v>
+      <c r="K60">
+        <v>0</v>
+      </c>
+      <c r="L60">
+        <v>6</v>
+      </c>
+      <c r="M60">
+        <v>3</v>
       </c>
       <c r="N60">
         <v>24</v>
       </c>
-      <c r="O60" s="6">
+      <c r="O60" s="5">
         <v>50.908000000000001</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B61" s="8">
+      <c r="B61" s="7">
         <v>2020</v>
       </c>
-      <c r="C61" s="9">
+      <c r="C61" s="8">
         <v>43891</v>
       </c>
-      <c r="D61" s="8" t="s">
+      <c r="D61" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E61" s="1" t="s">
@@ -3595,39 +3934,45 @@
       <c r="I61" s="3">
         <v>22.019178082191782</v>
       </c>
-      <c r="J61" s="7">
-        <v>3</v>
-      </c>
-      <c r="K61" s="4">
-        <v>0</v>
+      <c r="J61" s="6">
+        <v>3</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+      <c r="L61">
+        <v>6</v>
+      </c>
+      <c r="M61">
+        <v>2</v>
       </c>
       <c r="N61">
         <v>20</v>
       </c>
-      <c r="O61" s="6">
+      <c r="O61" s="5">
         <v>50.908000000000001</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A62" s="15" t="s">
+      <c r="A62" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B62" s="15">
+      <c r="B62" s="13">
         <v>2020</v>
       </c>
       <c r="C62" s="2">
         <v>43856</v>
       </c>
-      <c r="D62" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E62" s="6" t="s">
+      <c r="D62" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F62" s="6" t="s">
+      <c r="F62" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="G62" s="6" t="s">
+      <c r="G62" s="5" t="s">
         <v>28</v>
       </c>
       <c r="H62" s="3">
@@ -3636,37 +3981,43 @@
       <c r="I62" s="3">
         <v>27.772602739726029</v>
       </c>
-      <c r="J62" s="7">
+      <c r="J62" s="6">
         <v>1</v>
       </c>
       <c r="K62">
         <v>0</v>
+      </c>
+      <c r="L62">
+        <v>8</v>
+      </c>
+      <c r="M62">
+        <v>4</v>
       </c>
       <c r="N62">
         <v>30</v>
       </c>
-      <c r="O62" s="26"/>
+      <c r="O62" s="24"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A63" s="15" t="s">
+      <c r="A63" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B63" s="15">
+      <c r="B63" s="13">
         <v>2020</v>
       </c>
       <c r="C63" s="2">
         <v>43856</v>
       </c>
-      <c r="D63" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E63" s="6" t="s">
+      <c r="D63" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E63" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F63" s="6" t="s">
+      <c r="F63" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G63" s="6" t="s">
+      <c r="G63" s="5" t="s">
         <v>16</v>
       </c>
       <c r="H63" s="3">
@@ -3675,37 +4026,43 @@
       <c r="I63" s="3">
         <v>24.224657534246575</v>
       </c>
-      <c r="J63" s="7">
+      <c r="J63" s="6">
         <v>2</v>
       </c>
       <c r="K63">
         <v>0</v>
+      </c>
+      <c r="L63">
+        <v>9</v>
+      </c>
+      <c r="M63">
+        <v>2</v>
       </c>
       <c r="N63">
         <v>28</v>
       </c>
-      <c r="O63" s="26"/>
+      <c r="O63" s="24"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A64" s="15" t="s">
+      <c r="A64" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B64" s="15">
+      <c r="B64" s="13">
         <v>2020</v>
       </c>
       <c r="C64" s="2">
         <v>43856</v>
       </c>
-      <c r="D64" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E64" s="6" t="s">
+      <c r="D64" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F64" s="6" t="s">
+      <c r="F64" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G64" s="6" t="s">
+      <c r="G64" s="5" t="s">
         <v>69</v>
       </c>
       <c r="H64" s="3">
@@ -3714,28 +4071,34 @@
       <c r="I64" s="3">
         <v>25.104109589041094</v>
       </c>
-      <c r="J64" s="7">
-        <v>3</v>
-      </c>
-      <c r="K64" s="4">
-        <v>0</v>
+      <c r="J64" s="6">
+        <v>3</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+      <c r="L64">
+        <v>9</v>
+      </c>
+      <c r="M64">
+        <v>2</v>
       </c>
       <c r="N64">
         <v>24</v>
       </c>
-      <c r="O64" s="26"/>
+      <c r="O64" s="24"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B65" s="15">
+      <c r="B65" s="13">
         <v>2019</v>
       </c>
       <c r="C65" s="2">
         <v>43814</v>
       </c>
-      <c r="D65" s="15" t="s">
+      <c r="D65" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E65" s="1" t="s">
@@ -3753,30 +4116,36 @@
       <c r="I65" s="3">
         <v>28.024657534246575</v>
       </c>
-      <c r="J65" s="7">
+      <c r="J65" s="6">
         <v>1</v>
       </c>
       <c r="K65">
         <v>20</v>
       </c>
+      <c r="L65">
+        <v>11</v>
+      </c>
+      <c r="M65">
+        <v>5</v>
+      </c>
       <c r="N65">
         <v>56</v>
       </c>
-      <c r="O65" s="26">
+      <c r="O65" s="24">
         <v>48.262</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A66" s="15" t="s">
+      <c r="A66" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B66" s="15">
+      <c r="B66" s="13">
         <v>2019</v>
       </c>
       <c r="C66" s="2">
         <v>43814</v>
       </c>
-      <c r="D66" s="15" t="s">
+      <c r="D66" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E66" s="1" t="s">
@@ -3794,30 +4163,36 @@
       <c r="I66" s="3">
         <v>19.898630136986302</v>
       </c>
-      <c r="J66" s="7">
+      <c r="J66" s="6">
         <v>2</v>
       </c>
       <c r="K66">
         <v>20</v>
       </c>
+      <c r="L66">
+        <v>8</v>
+      </c>
+      <c r="M66">
+        <v>2</v>
+      </c>
       <c r="N66">
         <v>51</v>
       </c>
-      <c r="O66" s="26">
+      <c r="O66" s="24">
         <v>48.262</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A67" s="15" t="s">
+      <c r="A67" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B67" s="15">
+      <c r="B67" s="13">
         <v>2019</v>
       </c>
       <c r="C67" s="2">
         <v>43814</v>
       </c>
-      <c r="D67" s="15" t="s">
+      <c r="D67" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E67" s="1" t="s">
@@ -3835,39 +4210,45 @@
       <c r="I67" s="3">
         <v>33.095890410958901</v>
       </c>
-      <c r="J67" s="7">
+      <c r="J67" s="6">
         <v>3</v>
       </c>
       <c r="K67">
         <v>20</v>
       </c>
+      <c r="L67">
+        <v>4</v>
+      </c>
+      <c r="M67">
+        <v>1</v>
+      </c>
       <c r="N67">
         <v>32</v>
       </c>
-      <c r="O67" s="26">
+      <c r="O67" s="24">
         <v>48.262</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A68" s="15" t="s">
+      <c r="A68" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B68" s="15">
+      <c r="B68" s="13">
         <v>2019</v>
       </c>
       <c r="C68" s="2">
         <v>43807</v>
       </c>
-      <c r="D68" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E68" s="6" t="s">
+      <c r="D68" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E68" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F68" s="6" t="s">
+      <c r="F68" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G68" s="6" t="s">
+      <c r="G68" s="5" t="s">
         <v>42</v>
       </c>
       <c r="H68" s="3">
@@ -3876,39 +4257,45 @@
       <c r="I68" s="3">
         <v>23.789041095890411</v>
       </c>
-      <c r="J68" s="7">
+      <c r="J68" s="6">
         <v>1</v>
       </c>
       <c r="K68">
         <v>0</v>
+      </c>
+      <c r="L68">
+        <v>10</v>
+      </c>
+      <c r="M68">
+        <v>6</v>
       </c>
       <c r="N68">
         <v>42</v>
       </c>
-      <c r="O68" s="26">
+      <c r="O68" s="24">
         <v>49.936</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A69" s="15" t="s">
+      <c r="A69" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B69" s="15">
+      <c r="B69" s="13">
         <v>2019</v>
       </c>
       <c r="C69" s="2">
         <v>43807</v>
       </c>
-      <c r="D69" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E69" s="6" t="s">
+      <c r="D69" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="F69" s="6" t="s">
+      <c r="F69" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="G69" s="6" t="s">
+      <c r="G69" s="5" t="s">
         <v>99</v>
       </c>
       <c r="H69" s="3">
@@ -3917,39 +4304,45 @@
       <c r="I69" s="3">
         <v>23.55890410958904</v>
       </c>
-      <c r="J69" s="7">
+      <c r="J69" s="6">
         <v>2</v>
       </c>
       <c r="K69">
         <v>0</v>
+      </c>
+      <c r="L69">
+        <v>11</v>
+      </c>
+      <c r="M69">
+        <v>1</v>
       </c>
       <c r="N69">
         <v>32</v>
       </c>
-      <c r="O69" s="26">
+      <c r="O69" s="24">
         <v>49.936</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A70" s="15" t="s">
+      <c r="A70" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B70" s="15">
+      <c r="B70" s="13">
         <v>2019</v>
       </c>
       <c r="C70" s="2">
         <v>43807</v>
       </c>
-      <c r="D70" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E70" s="6" t="s">
+      <c r="D70" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E70" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F70" s="6" t="s">
+      <c r="F70" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G70" s="6" t="s">
+      <c r="G70" s="5" t="s">
         <v>122</v>
       </c>
       <c r="H70" s="3">
@@ -3958,16 +4351,22 @@
       <c r="I70" s="3">
         <v>23.147945205479452</v>
       </c>
-      <c r="J70" s="7">
+      <c r="J70" s="6">
         <v>3</v>
       </c>
       <c r="K70">
         <v>0</v>
+      </c>
+      <c r="L70">
+        <v>6</v>
+      </c>
+      <c r="M70">
+        <v>1</v>
       </c>
       <c r="N70">
         <v>19</v>
       </c>
-      <c r="O70" s="26">
+      <c r="O70" s="24">
         <v>49.936</v>
       </c>
     </row>
@@ -3999,16 +4398,22 @@
       <c r="I71" s="3">
         <v>31.512328767123286</v>
       </c>
-      <c r="J71" s="7">
+      <c r="J71" s="6">
         <v>1</v>
       </c>
       <c r="K71">
         <v>0</v>
+      </c>
+      <c r="L71">
+        <v>8</v>
+      </c>
+      <c r="M71">
+        <v>3</v>
       </c>
       <c r="N71">
         <v>31</v>
       </c>
-      <c r="O71" s="26">
+      <c r="O71" s="24">
         <v>40.737000000000002</v>
       </c>
     </row>
@@ -4040,16 +4445,22 @@
       <c r="I72" s="3">
         <v>23.12876712328767</v>
       </c>
-      <c r="J72" s="7">
+      <c r="J72" s="6">
         <v>2</v>
       </c>
-      <c r="K72" s="4">
-        <v>0</v>
+      <c r="K72">
+        <v>0</v>
+      </c>
+      <c r="L72">
+        <v>5</v>
+      </c>
+      <c r="M72">
+        <v>3</v>
       </c>
       <c r="N72">
         <v>24</v>
       </c>
-      <c r="O72" s="26">
+      <c r="O72" s="24">
         <v>40.737000000000002</v>
       </c>
     </row>
@@ -4081,39 +4492,45 @@
       <c r="I73" s="3">
         <v>20.449315068493149</v>
       </c>
-      <c r="J73" s="7">
-        <v>3</v>
-      </c>
-      <c r="K73" s="4">
-        <v>0</v>
+      <c r="J73" s="6">
+        <v>3</v>
+      </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
+      <c r="L73">
+        <v>6</v>
+      </c>
+      <c r="M73">
+        <v>2</v>
       </c>
       <c r="N73">
         <v>18</v>
       </c>
-      <c r="O73" s="26">
+      <c r="O73" s="24">
         <v>40.737000000000002</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A74" s="8" t="s">
+      <c r="A74" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B74" s="8">
+      <c r="B74" s="7">
         <v>2019</v>
       </c>
-      <c r="C74" s="9">
+      <c r="C74" s="8">
         <v>43777</v>
       </c>
-      <c r="D74" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E74" s="6" t="s">
+      <c r="D74" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F74" s="6" t="s">
+      <c r="F74" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G74" s="6" t="s">
+      <c r="G74" s="5" t="s">
         <v>42</v>
       </c>
       <c r="H74" s="3">
@@ -4122,39 +4539,45 @@
       <c r="I74" s="3">
         <v>25.153424657534245</v>
       </c>
-      <c r="J74" s="7">
+      <c r="J74" s="6">
         <v>1</v>
       </c>
       <c r="K74">
         <v>0</v>
+      </c>
+      <c r="L74">
+        <v>9</v>
+      </c>
+      <c r="M74">
+        <v>6</v>
       </c>
       <c r="N74">
         <v>40</v>
       </c>
-      <c r="O74" s="26">
+      <c r="O74" s="24">
         <v>52.779000000000003</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A75" s="8" t="s">
+      <c r="A75" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B75" s="8">
+      <c r="B75" s="7">
         <v>2019</v>
       </c>
-      <c r="C75" s="9">
+      <c r="C75" s="8">
         <v>43777</v>
       </c>
-      <c r="D75" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E75" s="6" t="s">
+      <c r="D75" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F75" s="6" t="s">
+      <c r="F75" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G75" s="6" t="s">
+      <c r="G75" s="5" t="s">
         <v>28</v>
       </c>
       <c r="H75" s="3">
@@ -4163,39 +4586,45 @@
       <c r="I75" s="3">
         <v>25.19178082191781</v>
       </c>
-      <c r="J75" s="7">
+      <c r="J75" s="6">
         <v>2</v>
       </c>
       <c r="K75">
         <v>0</v>
+      </c>
+      <c r="L75">
+        <v>6</v>
+      </c>
+      <c r="M75">
+        <v>5</v>
       </c>
       <c r="N75">
         <v>31</v>
       </c>
-      <c r="O75" s="26">
+      <c r="O75" s="24">
         <v>52.779000000000003</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B76" s="8">
+      <c r="B76" s="7">
         <v>2019</v>
       </c>
-      <c r="C76" s="9">
+      <c r="C76" s="8">
         <v>43777</v>
       </c>
-      <c r="D76" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E76" s="6" t="s">
+      <c r="D76" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F76" s="6" t="s">
+      <c r="F76" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G76" s="6" t="s">
+      <c r="G76" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H76" s="3">
@@ -4204,30 +4633,36 @@
       <c r="I76" s="3">
         <v>28.463013698630139</v>
       </c>
-      <c r="J76" s="7">
+      <c r="J76" s="6">
         <v>3</v>
       </c>
       <c r="K76">
+        <v>0</v>
+      </c>
+      <c r="L76">
+        <v>8</v>
+      </c>
+      <c r="M76">
         <v>0</v>
       </c>
       <c r="N76">
         <v>19</v>
       </c>
-      <c r="O76" s="26">
+      <c r="O76" s="24">
         <v>52.779000000000003</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A77" s="15" t="s">
+      <c r="A77" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B77" s="15">
+      <c r="B77" s="13">
         <v>2019</v>
       </c>
       <c r="C77" s="2">
         <v>43772</v>
       </c>
-      <c r="D77" s="15" t="s">
+      <c r="D77" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E77" s="1" t="s">
@@ -4245,30 +4680,36 @@
       <c r="I77" s="3">
         <v>28.44109589041096</v>
       </c>
-      <c r="J77" s="7">
+      <c r="J77" s="6">
         <v>1</v>
       </c>
       <c r="K77">
         <v>20</v>
       </c>
+      <c r="L77">
+        <v>10</v>
+      </c>
+      <c r="M77">
+        <v>3</v>
+      </c>
       <c r="N77">
         <v>50</v>
       </c>
-      <c r="O77" s="26">
+      <c r="O77" s="24">
         <v>53.268000000000001</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A78" s="15" t="s">
+      <c r="A78" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B78" s="15">
+      <c r="B78" s="13">
         <v>2019</v>
       </c>
       <c r="C78" s="2">
         <v>43772</v>
       </c>
-      <c r="D78" s="15" t="s">
+      <c r="D78" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E78" s="1" t="s">
@@ -4286,30 +4727,36 @@
       <c r="I78" s="3">
         <v>22.991780821917807</v>
       </c>
-      <c r="J78" s="7">
+      <c r="J78" s="6">
         <v>2</v>
       </c>
       <c r="K78">
         <v>20</v>
       </c>
+      <c r="L78">
+        <v>7</v>
+      </c>
+      <c r="M78">
+        <v>3</v>
+      </c>
       <c r="N78">
         <v>44</v>
       </c>
-      <c r="O78" s="26">
+      <c r="O78" s="24">
         <v>53.268000000000001</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A79" s="15" t="s">
+      <c r="A79" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B79" s="15">
+      <c r="B79" s="13">
         <v>2019</v>
       </c>
       <c r="C79" s="2">
         <v>43772</v>
       </c>
-      <c r="D79" s="15" t="s">
+      <c r="D79" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E79" s="1" t="s">
@@ -4327,16 +4774,22 @@
       <c r="I79" s="3">
         <v>19.783561643835615</v>
       </c>
-      <c r="J79" s="7">
+      <c r="J79" s="6">
         <v>3</v>
       </c>
       <c r="K79">
         <v>20</v>
       </c>
+      <c r="L79">
+        <v>5</v>
+      </c>
+      <c r="M79">
+        <v>1</v>
+      </c>
       <c r="N79">
         <v>35</v>
       </c>
-      <c r="O79" s="26">
+      <c r="O79" s="24">
         <v>53.268000000000001</v>
       </c>
     </row>
@@ -4344,22 +4797,22 @@
       <c r="A80" t="s">
         <v>45</v>
       </c>
-      <c r="B80" s="15">
+      <c r="B80" s="13">
         <v>2019</v>
       </c>
       <c r="C80" s="2">
         <v>43527</v>
       </c>
-      <c r="D80" s="15" t="s">
+      <c r="D80" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E80" s="6" t="s">
+      <c r="E80" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F80" s="6" t="s">
+      <c r="F80" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G80" s="6" t="s">
+      <c r="G80" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H80" s="3">
@@ -4368,16 +4821,22 @@
       <c r="I80" s="3">
         <v>27.769863013698629</v>
       </c>
-      <c r="J80" s="7">
+      <c r="J80" s="6">
         <v>1</v>
       </c>
       <c r="K80">
         <v>0</v>
+      </c>
+      <c r="L80">
+        <v>9</v>
+      </c>
+      <c r="M80">
+        <v>3</v>
       </c>
       <c r="N80">
         <v>33</v>
       </c>
-      <c r="O80" s="26">
+      <c r="O80" s="24">
         <v>42.21</v>
       </c>
     </row>
@@ -4385,22 +4844,22 @@
       <c r="A81" t="s">
         <v>45</v>
       </c>
-      <c r="B81" s="15">
+      <c r="B81" s="13">
         <v>2019</v>
       </c>
       <c r="C81" s="2">
         <v>43527</v>
       </c>
-      <c r="D81" s="15" t="s">
+      <c r="D81" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E81" s="6" t="s">
+      <c r="E81" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F81" s="6" t="s">
+      <c r="F81" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G81" s="6" t="s">
+      <c r="G81" s="5" t="s">
         <v>42</v>
       </c>
       <c r="H81" s="3">
@@ -4409,16 +4868,22 @@
       <c r="I81" s="3">
         <v>26.183561643835617</v>
       </c>
-      <c r="J81" s="7">
+      <c r="J81" s="6">
         <v>2</v>
       </c>
       <c r="K81">
         <v>0</v>
+      </c>
+      <c r="L81">
+        <v>9</v>
+      </c>
+      <c r="M81">
+        <v>4</v>
       </c>
       <c r="N81">
         <v>31</v>
       </c>
-      <c r="O81" s="26">
+      <c r="O81" s="24">
         <v>42.21</v>
       </c>
     </row>
@@ -4426,22 +4891,22 @@
       <c r="A82" t="s">
         <v>45</v>
       </c>
-      <c r="B82" s="15">
+      <c r="B82" s="13">
         <v>2019</v>
       </c>
       <c r="C82" s="2">
         <v>43527</v>
       </c>
-      <c r="D82" s="15" t="s">
+      <c r="D82" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="E82" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F82" s="6" t="s">
+      <c r="F82" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G82" s="6" t="s">
+      <c r="G82" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H82" s="3">
@@ -4450,16 +4915,22 @@
       <c r="I82" s="3">
         <v>26.652054794520549</v>
       </c>
-      <c r="J82" s="7">
+      <c r="J82" s="6">
         <v>3</v>
       </c>
       <c r="K82">
         <v>0</v>
+      </c>
+      <c r="L82">
+        <v>6</v>
+      </c>
+      <c r="M82">
+        <v>2</v>
       </c>
       <c r="N82">
         <v>24</v>
       </c>
-      <c r="O82" s="26">
+      <c r="O82" s="24">
         <v>42.21</v>
       </c>
     </row>
@@ -4467,13 +4938,13 @@
       <c r="A83" t="s">
         <v>25</v>
       </c>
-      <c r="B83" s="15">
+      <c r="B83" s="13">
         <v>2019</v>
       </c>
       <c r="C83" s="2">
         <v>43492</v>
       </c>
-      <c r="D83" s="15" t="s">
+      <c r="D83" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E83" s="1" t="s">
@@ -4491,16 +4962,22 @@
       <c r="I83" s="3">
         <v>27.673972602739727</v>
       </c>
-      <c r="J83" s="7">
+      <c r="J83" s="6">
         <v>1</v>
       </c>
-      <c r="K83" s="4">
-        <v>0</v>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83">
+        <v>7</v>
+      </c>
+      <c r="M83">
+        <v>4</v>
       </c>
       <c r="N83">
         <v>29</v>
       </c>
-      <c r="O83" s="26">
+      <c r="O83" s="24">
         <v>51.688000000000002</v>
       </c>
     </row>
@@ -4508,13 +4985,13 @@
       <c r="A84" t="s">
         <v>25</v>
       </c>
-      <c r="B84" s="15">
+      <c r="B84" s="13">
         <v>2019</v>
       </c>
       <c r="C84" s="2">
         <v>43492</v>
       </c>
-      <c r="D84" s="15" t="s">
+      <c r="D84" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E84" s="1" t="s">
@@ -4532,16 +5009,22 @@
       <c r="I84" s="3">
         <v>28.890410958904109</v>
       </c>
-      <c r="J84" s="7">
+      <c r="J84" s="6">
         <v>2</v>
       </c>
       <c r="K84">
         <v>0</v>
+      </c>
+      <c r="L84">
+        <v>8</v>
+      </c>
+      <c r="M84">
+        <v>1</v>
       </c>
       <c r="N84">
         <v>24</v>
       </c>
-      <c r="O84" s="26">
+      <c r="O84" s="24">
         <v>51.688000000000002</v>
       </c>
     </row>
@@ -4549,13 +5032,13 @@
       <c r="A85" t="s">
         <v>25</v>
       </c>
-      <c r="B85" s="15">
+      <c r="B85" s="13">
         <v>2019</v>
       </c>
       <c r="C85" s="2">
         <v>43492</v>
       </c>
-      <c r="D85" s="15" t="s">
+      <c r="D85" s="13" t="s">
         <v>14</v>
       </c>
       <c r="E85" s="1" t="s">
@@ -4573,16 +5056,22 @@
       <c r="I85" s="3">
         <v>25.843835616438355</v>
       </c>
-      <c r="J85" s="7">
-        <v>3</v>
-      </c>
-      <c r="K85" s="4">
-        <v>0</v>
+      <c r="J85" s="6">
+        <v>3</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85">
+        <v>4</v>
+      </c>
+      <c r="M85">
+        <v>1</v>
       </c>
       <c r="N85">
         <v>12</v>
       </c>
-      <c r="O85" s="26">
+      <c r="O85" s="24">
         <v>51.688000000000002</v>
       </c>
     </row>
@@ -4618,46 +5107,46 @@
       <formula>#REF!="Q"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J65">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="between">
+      <formula>0</formula>
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K68:K70">
-    <cfRule type="cellIs" dxfId="8" priority="19" operator="between">
+    <cfRule type="cellIs" dxfId="7" priority="19" operator="between">
       <formula>1</formula>
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="20" operator="between">
+    <cfRule type="cellIs" dxfId="6" priority="20" operator="between">
       <formula>2</formula>
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="21" operator="between">
+    <cfRule type="cellIs" dxfId="5" priority="21" operator="between">
       <formula>3</formula>
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="22" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="22" operator="between">
       <formula>5</formula>
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N68:N70">
-    <cfRule type="cellIs" dxfId="4" priority="23" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="23" operator="between">
       <formula>2</formula>
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="24" operator="between">
+    <cfRule type="cellIs" dxfId="2" priority="24" operator="between">
       <formula>4</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="25" operator="between">
+    <cfRule type="cellIs" dxfId="1" priority="25" operator="between">
       <formula>6</formula>
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="26" operator="between">
+    <cfRule type="cellIs" dxfId="0" priority="26" operator="between">
       <formula>10</formula>
       <formula>10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J65">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
-      <formula>0</formula>
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>